<commit_message>
File initial level-design findings for Nouraajd quests/dialog
First review-pass output from the level-designer loop, filed into the dedicated
worksheet via scripts/issue_queue.py propose (queue validation clean):

- [EPIC_60][STORY_01][SUBSTORY_01] holyRelic "only tool that can cleanse"
  description contradicts the OctoBogz contract completing without the relic (P1)
- [EPIC_60][STORY_01][SUBSTORY_02] OctoBogz cave biome continuity: dialog says
  desert/sand, surrounding signposts say swamp/mire (P2)
- [EPIC_60][STORY_01][SUBSTORY_03] RetrieveRelicQuest reward text vaguer than the
  concrete greater-potion unlock it grants (P2)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QsMo9ToVEYtjfbvyKx2XLj
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -31,7 +31,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:dimension ref="A1:AC1"/>
+  <x:dimension ref="A1:AC4"/>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
@@ -122,6 +122,245 @@
         <x:v>Attempt</x:v>
       </x:c>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>[EPIC_60][STORY_01][SUBSTORY_01]Holy relic description claims exclusive cleanse but OctoBogz contract completes without it</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>STORY_01</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>Quests and Dialog</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>SUBSTORY_01</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>Holy relic exclusivity contradiction</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>Bug</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>Level Design / Quests</x:v>
+      </x:c>
+      <x:c r="K2"/>
+      <x:c r="L2" t="str">
+        <x:v>res/maps/nouraajd/config.json
+res/maps/nouraajd/script.py</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>The holyRelic item description in res/maps/nouraajd/config.json reads 'A sanctified shard taken from the ruined chapel, the only tool that can cleanse the OctoBogz lair.' but the OctoBogz extermination contract completes without the relic. The onDestroy trigger for cave2 (res/maps/nouraajd/script.py:621-636 OctoBogzCaveTrigger) calls mark_octobogz_slain() and complete_octobogz_contract() unconditionally, granting the octoBogzQuest reward (1000 gold + ShadowBlade, OctoBogzQuest.onComplete). The RELIC_RETURNED check only gates the OCTOBOGZ_CLEARED flag and a flavor message (lines 631-636). A player can fully clear and be rewarded for the OctoBogz lair without ever obtaining the relic, contradicting the description's 'only tool' claim.</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>Description and mechanics agree: either (a) gate cave2 destruction/contract completion on RELIC_RETURNED so the relic is genuinely required, or (b) revise the holyRelic description to drop the exclusivity wording (e.g. 'blessed to purify the lair after the OctoBogz fall'). scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/maps/nouraajd/script.py</x:v>
+      </x:c>
+      <x:c r="Q2" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R2" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S2" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T2" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U2"/>
+      <x:c r="V2"/>
+      <x:c r="W2"/>
+      <x:c r="X2"/>
+      <x:c r="Y2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z2" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA2" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB2" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>[EPIC_60][STORY_01][SUBSTORY_02]OctoBogz cave described as desert sand in dialog but framed as swamp mire by surrounding signposts</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>STORY_01</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>Quests and Dialog</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>SUBSTORY_02</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>OctoBogz biome continuity</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>Bug</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>Level Design / Quests</x:v>
+      </x:c>
+      <x:c r="K3"/>
+      <x:c r="L3" t="str">
+        <x:v>res/maps/nouraajd/dialog2.json
+res/maps/nouraajd/config.json</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>The OctoBogz refugee dialog (res/maps/nouraajd/dialog2.json) repeatedly frames the cave as desert/sand: ASK_WHY 'leave bones in the sand', ASK_ABOUT_OCTOBOGZ 'ambushing from stone and sand alike', ACCEPT_QUEST 'half-buried under boulders and sand'. But the authored ambient signposts tied to the same OctoBogz/relic plot describe a swamp/mire biome: ambientSwampFisherWarning text 'FISHER WARNING - The mire keeps nets, names, and fingers...', ambientMireLantern 'A drowned lantern burns under the swamp skin...', ambientSwampReturnScratch 'Return the relic before the mire learns your name.' Two authored sources describe the same destination as incompatible biomes (desert vs swamp). The OctoBogz are described as part octopus, consistent with the swamp framing.</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>Biome wording is consistent for the OctoBogz lair: update the dialog2.json sand/desert phrasing to mire/marsh language (or vice versa) so dialog and ambient signposts agree. scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/maps/nouraajd/dialog2.json</x:v>
+      </x:c>
+      <x:c r="Q3" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R3" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S3" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T3" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U3"/>
+      <x:c r="V3"/>
+      <x:c r="W3"/>
+      <x:c r="X3"/>
+      <x:c r="Y3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z3" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA3" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB3" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>[EPIC_60][STORY_01][SUBSTORY_03]RetrieveRelicQuest reward text vaguer than the concrete greater-potion unlock it grants</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>STORY_01</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Quests and Dialog</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>SUBSTORY_03</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>Relic quest reward wording precision</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Improvement</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>Level Design / Quests</x:v>
+      </x:c>
+      <x:c r="K4"/>
+      <x:c r="L4" t="str">
+        <x:v>res/maps/nouraajd/script.py</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>RetrieveRelicQuest.getReward (res/maps/nouraajd/script.py:484) returns 'Unlocks stronger alchemy recipes.', but the actual grant is narrower and specific: BerenDialog.return_relic (script.py:906) sets CAN_BREW_GREATER_POTIONS, which res/config/crafting.json / res/plugins/crafting.py describe as greater-potion brewing only. The sibling DeliverLetterQuest.getReward ('Unlocks scribe-desk scroll crafting.') is precise about its CAN_CRAFT_SCROLLS unlock; the relic reward wording is comparatively vague and may lead players to expect new alchemy recipes beyond potions. The unlock fires correctly; only the player-facing text is loose.</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>RetrieveRelicQuest reward text names the concrete unlock, e.g. 'Unlocks greater potion brewing at the alchemy table.', matching CAN_BREW_GREATER_POTIONS. scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/maps/nouraajd/script.py</x:v>
+      </x:c>
+      <x:c r="Q4" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R4" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S4" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T4" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U4"/>
+      <x:c r="V4"/>
+      <x:c r="W4"/>
+      <x:c r="X4"/>
+      <x:c r="Y4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z4" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA4" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB4" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
File level-design economy finding for Victor reward market
Review cycle 2 (economy/balance lens). The economy is otherwise strongly
consistent with docs/nouraajd-economy.md; the one confirmable content
inconsistency:

- [EPIC_60][STORY_02][SUBSTORY_01] victorMarket redundantly stocks the Lesser
  potions already sold at the general market, diluting its documented
  "stronger potions reserved for Victor's reward market" intent (P2)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QsMo9ToVEYtjfbvyKx2XLj
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -31,7 +31,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:dimension ref="A1:AC4"/>
+  <x:dimension ref="A1:AC5"/>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
@@ -361,6 +361,85 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>[EPIC_60][STORY_02][SUBSTORY_01]Victor reward market redundantly stocks lesser potions already sold at the general market</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>STORY_02</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Encounters and Balance</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>SUBSTORY_01</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>Victor reward market potion redundancy</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Improvement</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>Level Design / Encounters</x:v>
+      </x:c>
+      <x:c r="K5"/>
+      <x:c r="L5" t="str">
+        <x:v>res/maps/nouraajd/config.json</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>docs/nouraajd-economy.md:10 states 'Stronger Life and Mana Potions are reserved for Victor's reward market after the courtyard rescue.', framing victorMarket as the home of the stronger potions. But victorMarket.properties.items (res/maps/nouraajd/config.json) lists LesserLifePotion, LifePotion, LesserManaPotion, ManaPotion -- it also stocks the two Lesser potions the player can already buy at exampleMarket (which lists LesserLifePotion and LesserManaPotion). This dilutes the reward market's intended 'stronger potions' identity; the Lesser entries are redundant. (Same default 400g price either way, so not exploitable -- purely a content/intent inconsistency.)</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>victorMarket.items contains only the stronger potions (LifePotion, ManaPotion), matching the 'stronger ... reserved for Victor's reward market' intent in docs/nouraajd-economy.md, with the redundant LesserLifePotion/LesserManaPotion entries removed. scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P5" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/docs/nouraajd-economy.md</x:v>
+      </x:c>
+      <x:c r="Q5" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R5" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S5" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T5" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U5"/>
+      <x:c r="V5"/>
+      <x:c r="W5"/>
+      <x:c r="X5"/>
+      <x:c r="Y5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z5" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA5" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB5" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
File level-design findings for siege and ritual maps
Review cycle 2 (other authored maps). Content logic across ritual/siege/
multilevel is otherwise clean; two confirmable hygiene/pacing improvements:

- [EPIC_60][STORY_04][SUBSTORY_01] siege defendSiegeQuest config carries dead
  objective/reward/hint keys shadowed by the Python getReward/getObjective/
  getHint overrides (CQuest prefers the override) (P2)
- [EPIC_60][STORY_02][SUBSTORY_02] ritual AnchorSanctumTrigger omits the
  spawn_wave call both other anchor triggers perform (pacing inconsistency) (P2)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QsMo9ToVEYtjfbvyKx2XLj
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -31,7 +31,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:dimension ref="A1:AC5"/>
+  <x:dimension ref="A1:AC7"/>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
@@ -440,6 +440,165 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>[EPIC_60][STORY_04][SUBSTORY_01]Siege quest config carries dead objective reward hint keys shadowed by Python overrides</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>STORY_04</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Content Integrity</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>SUBSTORY_01</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>Siege quest dead config strings</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Improvement</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>Level Design / Content</x:v>
+      </x:c>
+      <x:c r="K6"/>
+      <x:c r="L6" t="str">
+        <x:v>res/maps/siege/config.json
+res/maps/siege/script.py</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>defendSiegeQuest.properties in res/maps/siege/config.json defines objective ('Seal every siege gate with charged wands.'), reward ('500 gold and campaign completion.'), and hint ('Pritz mages carry extra wands.'). But DefendSiegeQuest in res/maps/siege/script.py (lines 50-58) overrides getObjective/getReward/getHint, and CQuest::getObjective/getReward/getHint (src/object/CQuest.cpp:38-60) return the Python override whenever one exists, falling back to the stored property only otherwise. So those three config strings are never read (dead data); only 'description' (not overridden) is used. No player-visible contradiction today because the values agree, but it is latent rot: a future edit to the config strings would have no effect and could silently diverge from the Python source of truth. The ritual map's quests already carry only 'description'.</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>defendSiegeQuest.properties contains only the keys actually consumed (description), with the dead objective/reward/hint keys removed so res/maps/siege/script.py is the single source of truth for that quest's player-facing text. scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/object/CQuest.cpp</x:v>
+      </x:c>
+      <x:c r="Q6" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R6" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S6" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T6" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U6"/>
+      <x:c r="V6"/>
+      <x:c r="W6"/>
+      <x:c r="X6"/>
+      <x:c r="Y6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z6" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA6" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB6" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>[EPIC_60][STORY_02][SUBSTORY_02]Ritual sanctum anchor trigger omits the spawn_wave call the other two anchors perform</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>STORY_02</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>Encounters and Balance</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>SUBSTORY_02</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>Ritual sanctum anchor missing defender wave</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Improvement</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>Level Design / Encounters</x:v>
+      </x:c>
+      <x:c r="K7"/>
+      <x:c r="L7" t="str">
+        <x:v>res/maps/ritual/script.py</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>In res/maps/ritual/script.py the three onDestroy anchor triggers are structurally identical except for one line: AnchorNorthTrigger (lines 286-297) and AnchorCryptTrigger (lines 299-310) both call spawn_wave(game_map) before update_anchor_progress(game_map), but AnchorSanctumTrigger (lines 312-322) omits spawn_wave entirely. Destroying the north or crypt anchor spawns a defender wave; destroying the sanctum anchor does not. The anchor count still increments and the ritual/leader logic still runs, so it is not a correctness bug, but it is an authored inconsistency in difficulty pacing across the three otherwise-identical anchors.</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>The sanctum anchor's defender-wave behavior is intentional and consistent: either add spawn_wave(game_map) to AnchorSanctumTrigger to match the north/crypt anchors, or, if the omission is deliberate (final anchor, no further wave wanted), add a brief comment documenting that intent. scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P7" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/maps/ritual/script.py</x:v>
+      </x:c>
+      <x:c r="Q7" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R7" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S7" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T7" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U7"/>
+      <x:c r="V7"/>
+      <x:c r="W7"/>
+      <x:c r="X7"/>
+      <x:c r="Y7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z7" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA7" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB7" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
File crafting/economy findings (failed-craft refund + money pump)
Resume review cycle (crafting/item content). Crafting recipes, unlock-flag
wiring, and item references are otherwise clean; two confirmable economy bugs
the content validator does not check:

- [EPIC_60][STORY_02][SUBSTORY_06] failed crafts return before consuming
  ingredients/gold (res/plugins/crafting.py:118-122), so successChance is a
  free retry (P1)
- [EPIC_60][STORY_02][SUBSTORY_07] crafting cheap low-power potions into a
  higher-power output and reselling nets positive gold (brew_mana_potion
  +460/cycle; full-potion chains ~+1600) -- re-verified against the CMarket
  buyback formula, correcting an earlier "no gold loop" note (P1)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QsMo9ToVEYtjfbvyKx2XLj
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -31,7 +31,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:dimension ref="A1:AC10"/>
+  <x:dimension ref="A1:AC12"/>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
@@ -838,6 +838,166 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>[EPIC_60][STORY_02][SUBSTORY_06]Failed crafts consume no ingredients or gold making success chance a free retry</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>STORY_02</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>Encounters and Balance</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>SUBSTORY_06</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Crafting failure refunds everything</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>Bug</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>Level Design / Economy</x:v>
+      </x:c>
+      <x:c r="K11"/>
+      <x:c r="L11" t="str">
+        <x:v>res/plugins/crafting.py
+res/config/crafting.json</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>In apply_recipe (res/plugins/crafting.py:109-126), the success-chance roll returns on failure BEFORE any cost is paid: line 118-120 'if success_chance &lt; 100 and randint(1,100) &gt; success_chance: return _status(False, "failed")', while remove_required_items(player, recipe[inputs]) and deduct_gold(player, recipe[gold]) are at lines 122-123 (success path only). So a failed craft consumes neither ingredients nor gold -- the player simply retries for free until success. This nullifies every recipe's successChance (brew_mana_potion 95, scribe_emergency_portal_scroll 85, blend_greater_* 90, etc. in res/config/crafting.json): there is no risk or reagent cost to failure, only a wasted turn. The user-facing failure message ('The reagents fizzled and nothing was created') implies the reagents should be lost.</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>A failed craft costs its reagents (and optionally the gold): move remove_required_items (at least the inputs) before the success-chance roll, or consume inputs on the failure path, so successChance is a real cost/risk. A focused test crafts a &lt;100% recipe enough times to observe ingredient loss on failure. scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/plugins/crafting.py</x:v>
+      </x:c>
+      <x:c r="Q11" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S11" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U11"/>
+      <x:c r="V11"/>
+      <x:c r="W11"/>
+      <x:c r="X11"/>
+      <x:c r="Y11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>[EPIC_60][STORY_02][SUBSTORY_07]Crafting cheap potions into higher-power ones and reselling is a repeatable gold exploit</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>STORY_02</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Encounters and Balance</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>SUBSTORY_07</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>Crafting-to-buyback money pump</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>Bug</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>Level Design / Economy</x:v>
+      </x:c>
+      <x:c r="K12"/>
+      <x:c r="L12" t="str">
+        <x:v>res/config/crafting.json
+res/config/potions.json</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>Several recipes turn cheap low-power inputs into a higher-power output whose vendor buyback exceeds total input cost, yielding repeatable profit. Market math (src/object/CMarket.cpp:35,43,138): price = 2^power*200 scaled by percent; player buys at sell%=100, sells back at getBuyCost = min(2^power*200*0.80, 5000) min'd with sellCost (CMarket.h:63-64). Worked example, brew_mana_potion (res/config/crafting.json): inputs 2x LesserManaPotion (potions.json power 1 -&gt; buy 400 each = 800) + 20 gold = 820 total; output ManaPotion (power 3) sells back for min(1600*0.8,5000)=1280. Net +460 per craft. LesserManaPotion is stocked (exampleMarket, victorMarket) and ManaPotion carries no 'quest' tag so it is sellable (CGameTradePanel blocks only Quest-tagged items). brew_full_life_potion / brew_full_mana_potion chains net ~+1600 (cheapest input cost ~3380/3460 vs 5000 capped buyback). The power jump (2x power-1 -&gt; power-3 for ManaPotion; 2x power-2 -&gt; power-3 GreaterLifePotion) is the root: it more than doubles value. NOTE: this contradicts an earlier review's 'no gold loop' note, which only considered buying and reselling the SAME item; the exploit is the crafting power-transformation, re-verified here against the CMarket formula. Compounded by the failed-craft-refund bug (no reagent cost on failure).</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>Total input value (ingredients + gold) is &gt;= output buyback for every craftable item, removing the positive-margin loop: lower the high output powers (ManaPotion power 3 and GreaterLifePotion power 3 are the anomalies vs their power-1/power-2 inputs), and/or raise the recipe gold costs, and/or reduce market buy%. Verify by computing buyback vs cheapest input cost for every recipe in crafting.json. scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O12" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P12" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/object/CMarket.cpp</x:v>
+      </x:c>
+      <x:c r="Q12" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S12" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U12"/>
+      <x:c r="V12"/>
+      <x:c r="W12"/>
+      <x:c r="X12"/>
+      <x:c r="Y12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Level-design review: file crafting/economy balance bugs (failed-craft refund + money pump) (#1047)
Resume review cycle (crafting/item content). Crafting recipes, unlock-flag
wiring, and item references are otherwise clean; two confirmable economy bugs
the content validator does not check:

- [EPIC_60][STORY_02][SUBSTORY_06] failed crafts return before consuming
  ingredients/gold (res/plugins/crafting.py:118-122), so successChance is a
  free retry (P1)
- [EPIC_60][STORY_02][SUBSTORY_07] crafting cheap low-power potions into a
  higher-power output and reselling nets positive gold (brew_mana_potion
  +460/cycle; full-potion chains ~+1600) -- re-verified against the CMarket
  buyback formula, correcting an earlier "no gold loop" note (P1)


Claude-Session: https://claude.ai/code/session_01QsMo9ToVEYtjfbvyKx2XLj

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -31,7 +31,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:dimension ref="A1:AC10"/>
+  <x:dimension ref="A1:AC12"/>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
@@ -838,6 +838,166 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>[EPIC_60][STORY_02][SUBSTORY_06]Failed crafts consume no ingredients or gold making success chance a free retry</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>STORY_02</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>Encounters and Balance</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>SUBSTORY_06</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Crafting failure refunds everything</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>Bug</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>Level Design / Economy</x:v>
+      </x:c>
+      <x:c r="K11"/>
+      <x:c r="L11" t="str">
+        <x:v>res/plugins/crafting.py
+res/config/crafting.json</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>In apply_recipe (res/plugins/crafting.py:109-126), the success-chance roll returns on failure BEFORE any cost is paid: line 118-120 'if success_chance &lt; 100 and randint(1,100) &gt; success_chance: return _status(False, "failed")', while remove_required_items(player, recipe[inputs]) and deduct_gold(player, recipe[gold]) are at lines 122-123 (success path only). So a failed craft consumes neither ingredients nor gold -- the player simply retries for free until success. This nullifies every recipe's successChance (brew_mana_potion 95, scribe_emergency_portal_scroll 85, blend_greater_* 90, etc. in res/config/crafting.json): there is no risk or reagent cost to failure, only a wasted turn. The user-facing failure message ('The reagents fizzled and nothing was created') implies the reagents should be lost.</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>A failed craft costs its reagents (and optionally the gold): move remove_required_items (at least the inputs) before the success-chance roll, or consume inputs on the failure path, so successChance is a real cost/risk. A focused test crafts a &lt;100% recipe enough times to observe ingredient loss on failure. scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/plugins/crafting.py</x:v>
+      </x:c>
+      <x:c r="Q11" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S11" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U11"/>
+      <x:c r="V11"/>
+      <x:c r="W11"/>
+      <x:c r="X11"/>
+      <x:c r="Y11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB11" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>[EPIC_60][STORY_02][SUBSTORY_07]Crafting cheap potions into higher-power ones and reselling is a repeatable gold exploit</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>EPIC_60</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Level Design Review</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>STORY_02</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Encounters and Balance</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>SUBSTORY_07</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>Crafting-to-buyback money pump</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>Bug</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>Level Design / Economy</x:v>
+      </x:c>
+      <x:c r="K12"/>
+      <x:c r="L12" t="str">
+        <x:v>res/config/crafting.json
+res/config/potions.json</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>Several recipes turn cheap low-power inputs into a higher-power output whose vendor buyback exceeds total input cost, yielding repeatable profit. Market math (src/object/CMarket.cpp:35,43,138): price = 2^power*200 scaled by percent; player buys at sell%=100, sells back at getBuyCost = min(2^power*200*0.80, 5000) min'd with sellCost (CMarket.h:63-64). Worked example, brew_mana_potion (res/config/crafting.json): inputs 2x LesserManaPotion (potions.json power 1 -&gt; buy 400 each = 800) + 20 gold = 820 total; output ManaPotion (power 3) sells back for min(1600*0.8,5000)=1280. Net +460 per craft. LesserManaPotion is stocked (exampleMarket, victorMarket) and ManaPotion carries no 'quest' tag so it is sellable (CGameTradePanel blocks only Quest-tagged items). brew_full_life_potion / brew_full_mana_potion chains net ~+1600 (cheapest input cost ~3380/3460 vs 5000 capped buyback). The power jump (2x power-1 -&gt; power-3 for ManaPotion; 2x power-2 -&gt; power-3 GreaterLifePotion) is the root: it more than doubles value. NOTE: this contradicts an earlier review's 'no gold loop' note, which only considered buying and reselling the SAME item; the exploit is the crafting power-transformation, re-verified here against the CMarket formula. Compounded by the failed-craft-refund bug (no reagent cost on failure).</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>Total input value (ingredients + gold) is &gt;= output buyback for every craftable item, removing the positive-margin loop: lower the high output powers (ManaPotion power 3 and GreaterLifePotion power 3 are the anomalies vs their power-1/power-2 inputs), and/or raise the recipe gold costs, and/or reduce market buy%. Verify by computing buyback vs cheapest input cost for every recipe in crafting.json. scripts/validate_content.py still passes.</x:v>
+      </x:c>
+      <x:c r="O12" t="str">
+        <x:v>python3 scripts/validate_content.py</x:v>
+      </x:c>
+      <x:c r="P12" t="str">
+        <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/object/CMarket.cpp</x:v>
+      </x:c>
+      <x:c r="Q12" t="str">
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="S12" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="T12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="U12"/>
+      <x:c r="V12"/>
+      <x:c r="W12"/>
+      <x:c r="X12"/>
+      <x:c r="Y12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AA12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AB12" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="AC12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete EPIC_60/STORY_02/SUBSTORY_03 OctoBogz balance (impl PR #1115)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -650,7 +650,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/config/monsters.json</x:v>
       </x:c>
       <x:c r="Q8" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R8" t="str">
         <x:v>controller/ctrl-vm-4078-31cf30b5/subagent-7</x:v>
@@ -665,20 +665,33 @@
         <x:v>2026-06-30T22:44:50Z</x:v>
       </x:c>
       <x:c r="V8" t="str">
-        <x:v>2026-06-30T22:44:50Z</x:v>
-      </x:c>
-      <x:c r="W8" t="str">
-        <x:v>2026-07-01T22:44:50Z</x:v>
-      </x:c>
-      <x:c r="X8"/>
+        <x:v>2026-06-30T23:06:45Z</x:v>
+      </x:c>
+      <x:c r="W8"/>
+      <x:c r="X8" t="str">
+        <x:v>2026-06-30T23:06:45Z</x:v>
+      </x:c>
       <x:c r="Y8" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z8" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4078-31cf30b5/subagent-7</x:v>
-      </x:c>
-      <x:c r="AA8"/>
-      <x:c r="AB8"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA8" t="str">
+        <x:v>Tuned cave2 OctoBogz early-fight difficulty. Reduced the dedicated OctoBogz template baseStats
+(dmgMin 17-&gt;12, dmgMax 21-&gt;16, stamina 10-&gt;7 =&gt; HP 91-&gt;70, dmg 16-21) and cave2 spawn count
+(5-&gt;3) for a fair early three-mob fight, within the level-design acceptance ranges. Scoped to the
+dedicated OctoBogz type + cave2 only; crit/hit/strength/IDs/animation preserved; baseline fixture
+regenerated. Delivered via impl PR #1115. The 'trivially skippable' aspect is structural engine
+behavior (Cave.onEnter spawn + removeObjectByName fires the completion onDestroy regardless of
+kills) requiring a design decision; reported as a noted follow-up (would break authored contract tests).</x:v>
+      </x:c>
+      <x:c r="AB8" t="str">
+        <x:v>GitHub Actions impl PR #1115 (head 04b03b6): linux, linux-fast, windows, windows-deps, validate,
+export all SUCCESS (linux-coverage non-required for this data change; full linux suite passed with
+no engine-test regression). tests.test_creature_stat_scale_baseline 4 OK; scripts/validate_content.py
+passed; JSON valid; git diff --check clean.</x:v>
+      </x:c>
       <x:c r="AC8" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_60/STORY_02/SUBSTORY_03 OctoBogz balance (impl PR #1115) (#1120)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -650,7 +650,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/config/monsters.json</x:v>
       </x:c>
       <x:c r="Q8" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R8" t="str">
         <x:v>controller/ctrl-vm-4078-31cf30b5/subagent-7</x:v>
@@ -665,20 +665,33 @@
         <x:v>2026-06-30T22:44:50Z</x:v>
       </x:c>
       <x:c r="V8" t="str">
-        <x:v>2026-06-30T22:44:50Z</x:v>
-      </x:c>
-      <x:c r="W8" t="str">
-        <x:v>2026-07-01T22:44:50Z</x:v>
-      </x:c>
-      <x:c r="X8"/>
+        <x:v>2026-06-30T23:06:45Z</x:v>
+      </x:c>
+      <x:c r="W8"/>
+      <x:c r="X8" t="str">
+        <x:v>2026-06-30T23:06:45Z</x:v>
+      </x:c>
       <x:c r="Y8" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z8" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4078-31cf30b5/subagent-7</x:v>
-      </x:c>
-      <x:c r="AA8"/>
-      <x:c r="AB8"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA8" t="str">
+        <x:v>Tuned cave2 OctoBogz early-fight difficulty. Reduced the dedicated OctoBogz template baseStats
+(dmgMin 17-&gt;12, dmgMax 21-&gt;16, stamina 10-&gt;7 =&gt; HP 91-&gt;70, dmg 16-21) and cave2 spawn count
+(5-&gt;3) for a fair early three-mob fight, within the level-design acceptance ranges. Scoped to the
+dedicated OctoBogz type + cave2 only; crit/hit/strength/IDs/animation preserved; baseline fixture
+regenerated. Delivered via impl PR #1115. The 'trivially skippable' aspect is structural engine
+behavior (Cave.onEnter spawn + removeObjectByName fires the completion onDestroy regardless of
+kills) requiring a design decision; reported as a noted follow-up (would break authored contract tests).</x:v>
+      </x:c>
+      <x:c r="AB8" t="str">
+        <x:v>GitHub Actions impl PR #1115 (head 04b03b6): linux, linux-fast, windows, windows-deps, validate,
+export all SUCCESS (linux-coverage non-required for this data change; full linux suite passed with
+no engine-test regression). tests.test_creature_stat_scale_baseline 4 OK; scripts/validate_content.py
+passed; JSON valid; git diff --check clean.</x:v>
+      </x:c>
       <x:c r="AC8" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_60/STORY_01/SUBSTORY_01 holy relic description (impl PR #1118)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -171,7 +171,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/maps/nouraajd/script.py</x:v>
       </x:c>
       <x:c r="Q2" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R2" t="str">
         <x:v>controller/ctrl-vm-4078-31cf30b5/subagent-9</x:v>
@@ -186,20 +186,33 @@
         <x:v>2026-06-30T22:52:55Z</x:v>
       </x:c>
       <x:c r="V2" t="str">
-        <x:v>2026-06-30T22:52:55Z</x:v>
-      </x:c>
-      <x:c r="W2" t="str">
-        <x:v>2026-07-01T22:52:55Z</x:v>
-      </x:c>
-      <x:c r="X2"/>
+        <x:v>2026-06-30T23:09:19Z</x:v>
+      </x:c>
+      <x:c r="W2"/>
+      <x:c r="X2" t="str">
+        <x:v>2026-06-30T23:09:19Z</x:v>
+      </x:c>
       <x:c r="Y2" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z2" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4078-31cf30b5/subagent-9</x:v>
-      </x:c>
-      <x:c r="AA2"/>
-      <x:c r="AB2"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA2" t="str">
+        <x:v>Aligned the holyRelic item description with the actual OctoBogz contract mechanics. The
+description claimed the relic was 'the only tool that can cleanse the OctoBogz lair', but the
+cave2 OctoBogzCaveTrigger completes the extermination contract unconditionally; RELIC_RETURNED
+only gates the OCTOBOGZ_CLEARED flag and a purification flavor message (the killed-without-relic
+path is intended and tested). Chose acceptance option (b): revised the description to drop the
+false exclusivity ('blessed to purify the OctoBogz lair once the brood has fallen'), matching the
+relic's real post-clear-purification role. Description-only; no contract/trigger behavior altered.
+Delivered via impl PR #1118.</x:v>
+      </x:c>
+      <x:c r="AB2" t="str">
+        <x:v>GitHub Actions impl PR #1118 (head): linux, linux-fast, windows, windows-deps, validate, export all
+SUCCESS (linux-coverage non-required for this content change; full linux suite passed - no test
+asserts the description string). scripts/validate_content.py passed; JSON valid; git diff --check clean.</x:v>
+      </x:c>
       <x:c r="AC2" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_60/STORY_01/SUBSTORY_01 holy relic description (impl PR #1118) (#1122)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -171,7 +171,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/maps/nouraajd/script.py</x:v>
       </x:c>
       <x:c r="Q2" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R2" t="str">
         <x:v>controller/ctrl-vm-4078-31cf30b5/subagent-9</x:v>
@@ -186,20 +186,33 @@
         <x:v>2026-06-30T22:52:55Z</x:v>
       </x:c>
       <x:c r="V2" t="str">
-        <x:v>2026-06-30T22:52:55Z</x:v>
-      </x:c>
-      <x:c r="W2" t="str">
-        <x:v>2026-07-01T22:52:55Z</x:v>
-      </x:c>
-      <x:c r="X2"/>
+        <x:v>2026-06-30T23:09:19Z</x:v>
+      </x:c>
+      <x:c r="W2"/>
+      <x:c r="X2" t="str">
+        <x:v>2026-06-30T23:09:19Z</x:v>
+      </x:c>
       <x:c r="Y2" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z2" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4078-31cf30b5/subagent-9</x:v>
-      </x:c>
-      <x:c r="AA2"/>
-      <x:c r="AB2"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA2" t="str">
+        <x:v>Aligned the holyRelic item description with the actual OctoBogz contract mechanics. The
+description claimed the relic was 'the only tool that can cleanse the OctoBogz lair', but the
+cave2 OctoBogzCaveTrigger completes the extermination contract unconditionally; RELIC_RETURNED
+only gates the OCTOBOGZ_CLEARED flag and a purification flavor message (the killed-without-relic
+path is intended and tested). Chose acceptance option (b): revised the description to drop the
+false exclusivity ('blessed to purify the OctoBogz lair once the brood has fallen'), matching the
+relic's real post-clear-purification role. Description-only; no contract/trigger behavior altered.
+Delivered via impl PR #1118.</x:v>
+      </x:c>
+      <x:c r="AB2" t="str">
+        <x:v>GitHub Actions impl PR #1118 (head): linux, linux-fast, windows, windows-deps, validate, export all
+SUCCESS (linux-coverage non-required for this content change; full linux suite passed - no test
+asserts the description string). scripts/validate_content.py passed; JSON valid; git diff --check clean.</x:v>
+      </x:c>
       <x:c r="AC2" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Block EPIC_60/STORY_02/SUBSTORY_07 crafting economy (engine-test reconciliation needs native env)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -999,7 +999,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/object/CMarket.cpp</x:v>
       </x:c>
       <x:c r="Q12" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="R12" t="str">
         <x:v>controller/ctrl-vm-4078-31cf30b5/subagent-8</x:v>
@@ -1014,20 +1014,41 @@
         <x:v>2026-06-30T22:52:14Z</x:v>
       </x:c>
       <x:c r="V12" t="str">
-        <x:v>2026-06-30T22:52:14Z</x:v>
-      </x:c>
-      <x:c r="W12" t="str">
-        <x:v>2026-07-01T22:52:14Z</x:v>
-      </x:c>
+        <x:v>2026-06-30T23:25:51Z</x:v>
+      </x:c>
+      <x:c r="W12"/>
       <x:c r="X12"/>
       <x:c r="Y12" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z12" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4078-31cf30b5/subagent-8</x:v>
-      </x:c>
-      <x:c r="AA12"/>
-      <x:c r="AB12"/>
+        <x:v>Economy fix conflicts with un-runnable/un-diagnosable engine crafting GameTests; needs native-test env or designer lever decision</x:v>
+      </x:c>
+      <x:c r="AA12" t="str">
+        <x:v>BLOCKED on native-test reconciliation. The economy analysis and fix are complete and correct at the
+data level: every craftable recipe is driven to vendor-buyback margin &lt;= 0 (verified by a new live
+invariant test tests/test_crafting_economy_no_profit.py and content_validator 111 OK). However, the
+fix cannot be landed because it repeatedly conflicts with engine-backed crafting GameTests in the
+native suite ("[test shard 2]") that THIS environment cannot run (no native _game module; submodules
+unfetchable) or diagnose (CI log retrieval returns only the cleanup tail, not the failing assertion):
+- Lever A (ManaPotion power 3-&gt;2): a real potency reduction (potion.py onUse addManaProc(power*20),
+  60-&gt;40 mana) that broke an engine GameTest asserting ManaPotion's mana/value. Reverted.
+- Lever B (raise brew_mana_potion gold 20-&gt;640): closes the +620 margin with zero potency change but
+  breaks a different engine crafting GameTest in shard 2 (specific assertion not extractable from the
+  tail-only CI log after 3 iterations).
+- The brew_full_{life,mana}_potion input swap (Greater-&gt;Max, no power change) appears test-safe and
+  fixes the two larger +2350 exploits.
+Resolution needs either a native-test-capable environment to run the failing GameTest and reconcile
+it precisely, or a designer decision on the preferred economy lever (gold vs power vs output count)
+and explicit approval to update the conflicting GameTest. Implementation PR #1119 (data + invariant
+test) is left as a starting point; do not merge until the engine test passes.</x:v>
+      </x:c>
+      <x:c r="AB12" t="str">
+        <x:v>Local validation that passed: tests.test_crafting_economy_no_profit (3 OK), tests.test_content_validator
+(111 OK), scripts/validate_content.py (passed), JSON valid, margin calc all &lt;=0, git diff --check clean.
+Blocking validation: native build workflow linux job FAILED across 3 attempts on an engine GameTest in
+"[test shard 2]" that cannot be run or diagnosed in this build-less environment.</x:v>
+      </x:c>
       <x:c r="AC12" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Block EPIC_60/STORY_02/SUBSTORY_07 crafting economy (engine-test reconciliation needs native env) (#1126)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -999,7 +999,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/object/CMarket.cpp</x:v>
       </x:c>
       <x:c r="Q12" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="R12" t="str">
         <x:v>controller/ctrl-vm-4078-31cf30b5/subagent-8</x:v>
@@ -1014,20 +1014,41 @@
         <x:v>2026-06-30T22:52:14Z</x:v>
       </x:c>
       <x:c r="V12" t="str">
-        <x:v>2026-06-30T22:52:14Z</x:v>
-      </x:c>
-      <x:c r="W12" t="str">
-        <x:v>2026-07-01T22:52:14Z</x:v>
-      </x:c>
+        <x:v>2026-06-30T23:25:51Z</x:v>
+      </x:c>
+      <x:c r="W12"/>
       <x:c r="X12"/>
       <x:c r="Y12" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z12" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4078-31cf30b5/subagent-8</x:v>
-      </x:c>
-      <x:c r="AA12"/>
-      <x:c r="AB12"/>
+        <x:v>Economy fix conflicts with un-runnable/un-diagnosable engine crafting GameTests; needs native-test env or designer lever decision</x:v>
+      </x:c>
+      <x:c r="AA12" t="str">
+        <x:v>BLOCKED on native-test reconciliation. The economy analysis and fix are complete and correct at the
+data level: every craftable recipe is driven to vendor-buyback margin &lt;= 0 (verified by a new live
+invariant test tests/test_crafting_economy_no_profit.py and content_validator 111 OK). However, the
+fix cannot be landed because it repeatedly conflicts with engine-backed crafting GameTests in the
+native suite ("[test shard 2]") that THIS environment cannot run (no native _game module; submodules
+unfetchable) or diagnose (CI log retrieval returns only the cleanup tail, not the failing assertion):
+- Lever A (ManaPotion power 3-&gt;2): a real potency reduction (potion.py onUse addManaProc(power*20),
+  60-&gt;40 mana) that broke an engine GameTest asserting ManaPotion's mana/value. Reverted.
+- Lever B (raise brew_mana_potion gold 20-&gt;640): closes the +620 margin with zero potency change but
+  breaks a different engine crafting GameTest in shard 2 (specific assertion not extractable from the
+  tail-only CI log after 3 iterations).
+- The brew_full_{life,mana}_potion input swap (Greater-&gt;Max, no power change) appears test-safe and
+  fixes the two larger +2350 exploits.
+Resolution needs either a native-test-capable environment to run the failing GameTest and reconcile
+it precisely, or a designer decision on the preferred economy lever (gold vs power vs output count)
+and explicit approval to update the conflicting GameTest. Implementation PR #1119 (data + invariant
+test) is left as a starting point; do not merge until the engine test passes.</x:v>
+      </x:c>
+      <x:c r="AB12" t="str">
+        <x:v>Local validation that passed: tests.test_crafting_economy_no_profit (3 OK), tests.test_content_validator
+(111 OK), scripts/validate_content.py (passed), JSON valid, margin calc all &lt;=0, git diff --check clean.
+Blocking validation: native build workflow linux job FAILED across 3 attempts on an engine GameTest in
+"[test shard 2]" that cannot be run or diagnosed in this build-less environment.</x:v>
+      </x:c>
       <x:c r="AC12" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_60/STORY_02/SUBSTORY_06 failed-craft cost (impl PR #1114)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -917,7 +917,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/plugins/crafting.py</x:v>
       </x:c>
       <x:c r="Q11" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R11" t="str">
         <x:v>controller/ctrl-vm-4078-31cf30b5/subagent-6</x:v>
@@ -932,20 +932,34 @@
         <x:v>2026-06-30T22:44:18Z</x:v>
       </x:c>
       <x:c r="V11" t="str">
-        <x:v>2026-06-30T22:44:18Z</x:v>
-      </x:c>
-      <x:c r="W11" t="str">
-        <x:v>2026-07-01T22:44:18Z</x:v>
-      </x:c>
-      <x:c r="X11"/>
+        <x:v>2026-06-30T23:32:34Z</x:v>
+      </x:c>
+      <x:c r="W11"/>
+      <x:c r="X11" t="str">
+        <x:v>2026-06-30T23:32:34Z</x:v>
+      </x:c>
       <x:c r="Y11" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z11" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4078-31cf30b5/subagent-6</x:v>
-      </x:c>
-      <x:c r="AA11"/>
-      <x:c r="AB11"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA11" t="str">
+        <x:v>Fixed the free-retry crafting exploit. apply_recipe (res/plugins/crafting.py) returned on the
+success-chance failure roll BEFORE paying any cost, so a failed craft consumed nothing. Hoisted
+remove_required_items + deduct_gold above the roll (after the existing inventory/gold precondition
+gates that still guard both paths), so a failed craft now costs its inputs and gold while withholding
+outputs; the success path is behaviorally unchanged. Added tests/regression/test_crafting_failure_cost.py
+(4 tests) and reconciled the existing test_crafting_transactions_are_atomic RNG-failure section to the
+corrected, still-atomic contract (verified no design-intent for free-on-failure; recipes' 95/90/85
+successChance values are only meaningful with a failure cost). Delivered via impl PR #1114.</x:v>
+      </x:c>
+      <x:c r="AB11" t="str">
+        <x:v>GitHub Actions impl PR #1114 (head 02ae980): linux, linux-fast, windows, windows-deps, linux-coverage,
+validate, export all SUCCESS (coverage required for the crafting.py code change; full native GameTest
+suite including the reconciled atomic test passed). Local: tests.regression.test_crafting_failure_cost
+4 OK (sensitivity-checked against pre-fix source); py_compile + git diff --check clean.</x:v>
+      </x:c>
       <x:c r="AC11" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_60/STORY_02/SUBSTORY_06 failed-craft cost (impl PR #1114) (#1128)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -917,7 +917,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/plugins/crafting.py</x:v>
       </x:c>
       <x:c r="Q11" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R11" t="str">
         <x:v>controller/ctrl-vm-4078-31cf30b5/subagent-6</x:v>
@@ -932,20 +932,34 @@
         <x:v>2026-06-30T22:44:18Z</x:v>
       </x:c>
       <x:c r="V11" t="str">
-        <x:v>2026-06-30T22:44:18Z</x:v>
-      </x:c>
-      <x:c r="W11" t="str">
-        <x:v>2026-07-01T22:44:18Z</x:v>
-      </x:c>
-      <x:c r="X11"/>
+        <x:v>2026-06-30T23:32:34Z</x:v>
+      </x:c>
+      <x:c r="W11"/>
+      <x:c r="X11" t="str">
+        <x:v>2026-06-30T23:32:34Z</x:v>
+      </x:c>
       <x:c r="Y11" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z11" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4078-31cf30b5/subagent-6</x:v>
-      </x:c>
-      <x:c r="AA11"/>
-      <x:c r="AB11"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA11" t="str">
+        <x:v>Fixed the free-retry crafting exploit. apply_recipe (res/plugins/crafting.py) returned on the
+success-chance failure roll BEFORE paying any cost, so a failed craft consumed nothing. Hoisted
+remove_required_items + deduct_gold above the roll (after the existing inventory/gold precondition
+gates that still guard both paths), so a failed craft now costs its inputs and gold while withholding
+outputs; the success path is behaviorally unchanged. Added tests/regression/test_crafting_failure_cost.py
+(4 tests) and reconciled the existing test_crafting_transactions_are_atomic RNG-failure section to the
+corrected, still-atomic contract (verified no design-intent for free-on-failure; recipes' 95/90/85
+successChance values are only meaningful with a failure cost). Delivered via impl PR #1114.</x:v>
+      </x:c>
+      <x:c r="AB11" t="str">
+        <x:v>GitHub Actions impl PR #1114 (head 02ae980): linux, linux-fast, windows, windows-deps, linux-coverage,
+validate, export all SUCCESS (coverage required for the crafting.py code change; full native GameTest
+suite including the reconciled atomic test passed). Local: tests.regression.test_crafting_failure_cost
+4 OK (sensitivity-checked against pre-fix source); py_compile + git diff --check clean.</x:v>
+      </x:c>
       <x:c r="AC11" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Fix ritual sanctum anchor omitting spawn_wave (E60/S02/SS02)
AnchorNorthTrigger and AnchorCryptTrigger both call spawn_wave(game_map)
when their anchor is destroyed, but AnchorSanctumTrigger omitted it,
breaking the parallel escalation the three anchors are meant to share.
Add the missing spawn_wave(game_map) call to AnchorSanctumTrigger so
destroying the sanctum anchor spawns a defensive wave like the other two.

Behavior-consistent, one-line fix; no id or trigger renames. No ritual
test counts wave monsters, so no test change is required.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVs74ScY29D4F63H4rT1t2
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -583,35 +583,41 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/maps/ritual/script.py</x:v>
       </x:c>
       <x:c r="Q7" t="str">
-        <x:v>NOT_STARTED</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R7" t="str">
-        <x:v/>
+        <x:v>controller/ctrl-vm-5484-a0eec458/subagent-ritualwave</x:v>
       </x:c>
       <x:c r="S7" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="T7" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="U7"/>
-      <x:c r="V7"/>
+        <x:v>87b96ef1-428c-4552-b9fc-f70e2f8230e3</x:v>
+      </x:c>
+      <x:c r="U7" t="str">
+        <x:v>2026-07-01T17:22:43Z</x:v>
+      </x:c>
+      <x:c r="V7" t="str">
+        <x:v>2026-07-01T17:23:21Z</x:v>
+      </x:c>
       <x:c r="W7"/>
-      <x:c r="X7"/>
+      <x:c r="X7" t="str">
+        <x:v>2026-07-01T17:23:21Z</x:v>
+      </x:c>
       <x:c r="Y7" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z7" t="str">
-        <x:v/>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="AA7" t="str">
-        <x:v/>
+        <x:v>Fixed the parallel-structure defect: AnchorSanctumTrigger.trigger now calls spawn_wave(game_map) between showMessage and update_anchor_progress, exactly like AnchorNorthTrigger and AnchorCryptTrigger. Destroying the sanctum anchor now spawns a defensive wave like the other two anchors, restoring consistent escalation. One-line addition; no id/behavior renames.</x:v>
       </x:c>
       <x:c r="AB7" t="str">
-        <x:v/>
+        <x:v>python ast parse OK; validate_content passes; no ritual test counts wave monsters (test_ritual_quest_requires_successful_disruption / test_ritual_happy_path_frees_captive_and_starts_siege assert only flags/gold/quests/transition), so behavior-consistent fix needs no test change. Full native CI (build + campaign gates + C++) to confirm the ritual walkthrough on merge.</x:v>
       </x:c>
       <x:c r="AC7" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
Fix ritual sanctum anchor omitting spawn_wave (E60/S02/SS02) (#1245)
AnchorNorthTrigger and AnchorCryptTrigger both call spawn_wave(game_map)
when their anchor is destroyed, but AnchorSanctumTrigger omitted it,
breaking the parallel escalation the three anchors are meant to share.
Add the missing spawn_wave(game_map) call to AnchorSanctumTrigger so
destroying the sanctum anchor spawns a defensive wave like the other two.

Behavior-consistent, one-line fix; no id or trigger renames. No ritual
test counts wave monsters, so no test change is required.


Claude-Session: https://claude.ai/code/session_01UVs74ScY29D4F63H4rT1t2

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -583,35 +583,41 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/res/maps/ritual/script.py</x:v>
       </x:c>
       <x:c r="Q7" t="str">
-        <x:v>NOT_STARTED</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R7" t="str">
-        <x:v/>
+        <x:v>controller/ctrl-vm-5484-a0eec458/subagent-ritualwave</x:v>
       </x:c>
       <x:c r="S7" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="T7" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="U7"/>
-      <x:c r="V7"/>
+        <x:v>87b96ef1-428c-4552-b9fc-f70e2f8230e3</x:v>
+      </x:c>
+      <x:c r="U7" t="str">
+        <x:v>2026-07-01T17:22:43Z</x:v>
+      </x:c>
+      <x:c r="V7" t="str">
+        <x:v>2026-07-01T17:23:21Z</x:v>
+      </x:c>
       <x:c r="W7"/>
-      <x:c r="X7"/>
+      <x:c r="X7" t="str">
+        <x:v>2026-07-01T17:23:21Z</x:v>
+      </x:c>
       <x:c r="Y7" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z7" t="str">
-        <x:v/>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="AA7" t="str">
-        <x:v/>
+        <x:v>Fixed the parallel-structure defect: AnchorSanctumTrigger.trigger now calls spawn_wave(game_map) between showMessage and update_anchor_progress, exactly like AnchorNorthTrigger and AnchorCryptTrigger. Destroying the sanctum anchor now spawns a defensive wave like the other two anchors, restoring consistent escalation. One-line addition; no id/behavior renames.</x:v>
       </x:c>
       <x:c r="AB7" t="str">
-        <x:v/>
+        <x:v>python ast parse OK; validate_content passes; no ritual test counts wave monsters (test_ritual_quest_requires_successful_disruption / test_ritual_happy_path_frees_captive_and_starts_siege assert only flags/gold/quests/transition), so behavior-consistent fix needs no test change. Full native CI (build + campaign gates + C++) to confirm the ritual walkthrough on merge.</x:v>
       </x:c>
       <x:c r="AC7" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
Remove dead objective/reward/hint keys from defendSiegeQuest config (E60/S04/SS01)
defendSiegeQuest.properties in res/maps/siege/config.json defined
objective/reward/hint strings that were never read: DefendSiegeQuest in
res/maps/siege/script.py overrides getObjective/getReward/getHint, and
CQuest::getObjective/getReward/getHint return the Python override whenever
one exists, falling back to the stored property only otherwise. Only
'description' (not overridden) was actually consumed.

Remove the three dead keys so script.py is the single source of truth for
that quest's player-facing text and a future config edit cannot silently
diverge. Values were identical, so this is behavior-preserving. The ritual
map's quests already carry only 'description'.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVs74ScY29D4F63H4rT1t2
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -504,35 +504,41 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/object/CQuest.cpp</x:v>
       </x:c>
       <x:c r="Q6" t="str">
-        <x:v>NOT_STARTED</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R6" t="str">
-        <x:v/>
+        <x:v>controller/ctrl-vm-5484-a0eec458/subagent-siegecfg</x:v>
       </x:c>
       <x:c r="S6" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="T6" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="U6"/>
-      <x:c r="V6"/>
+        <x:v>7ac48f0a-5625-4e21-8541-38f0ab0261ec</x:v>
+      </x:c>
+      <x:c r="U6" t="str">
+        <x:v>2026-07-01T17:53:13Z</x:v>
+      </x:c>
+      <x:c r="V6" t="str">
+        <x:v>2026-07-01T17:53:58Z</x:v>
+      </x:c>
       <x:c r="W6"/>
-      <x:c r="X6"/>
+      <x:c r="X6" t="str">
+        <x:v>2026-07-01T17:53:58Z</x:v>
+      </x:c>
       <x:c r="Y6" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z6" t="str">
-        <x:v/>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="AA6" t="str">
-        <x:v/>
+        <x:v>Removed the dead objective/reward/hint keys from defendSiegeQuest.properties in res/maps/siege/config.json, leaving only the consumed 'description'. DefendSiegeQuest in siege/script.py overrides getObjective/getReward/getHint, and CQuest returns the Python override whenever one exists, so those three config strings were never read. res/maps/siege/script.py is now the single source of truth for that quest's objective/reward/hint text. Values were identical, so no player-visible change. Behavior-preserving.</x:v>
       </x:c>
       <x:c r="AB6" t="str">
-        <x:v/>
+        <x:v>python json parse OK; validate_content passes (siege map still valid); no test references the removed config keys. Native campaign gate (siege walkthrough) confirms on CI.</x:v>
       </x:c>
       <x:c r="AC6" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>

<commit_message>
Remove dead objective/reward/hint keys from defendSiegeQuest config (E60/S04/SS01) (#1246)
defendSiegeQuest.properties in res/maps/siege/config.json defined
objective/reward/hint strings that were never read: DefendSiegeQuest in
res/maps/siege/script.py overrides getObjective/getReward/getHint, and
CQuest::getObjective/getReward/getHint return the Python override whenever
one exists, falling back to the stored property only otherwise. Only
'description' (not overridden) was actually consumed.

Remove the three dead keys so script.py is the single source of truth for
that quest's player-facing text and a future config edit cannot silently
diverge. Values were identical, so this is behavior-preserving. The ritual
map's quests already carry only 'description'.


Claude-Session: https://claude.ai/code/session_01UVs74ScY29D4F63H4rT1t2

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -504,35 +504,41 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/object/CQuest.cpp</x:v>
       </x:c>
       <x:c r="Q6" t="str">
-        <x:v>NOT_STARTED</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R6" t="str">
-        <x:v/>
+        <x:v>controller/ctrl-vm-5484-a0eec458/subagent-siegecfg</x:v>
       </x:c>
       <x:c r="S6" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="T6" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="U6"/>
-      <x:c r="V6"/>
+        <x:v>7ac48f0a-5625-4e21-8541-38f0ab0261ec</x:v>
+      </x:c>
+      <x:c r="U6" t="str">
+        <x:v>2026-07-01T17:53:13Z</x:v>
+      </x:c>
+      <x:c r="V6" t="str">
+        <x:v>2026-07-01T17:53:58Z</x:v>
+      </x:c>
       <x:c r="W6"/>
-      <x:c r="X6"/>
+      <x:c r="X6" t="str">
+        <x:v>2026-07-01T17:53:58Z</x:v>
+      </x:c>
       <x:c r="Y6" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z6" t="str">
-        <x:v/>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="AA6" t="str">
-        <x:v/>
+        <x:v>Removed the dead objective/reward/hint keys from defendSiegeQuest.properties in res/maps/siege/config.json, leaving only the consumed 'description'. DefendSiegeQuest in siege/script.py overrides getObjective/getReward/getHint, and CQuest returns the Python override whenever one exists, so those three config strings were never read. res/maps/siege/script.py is now the single source of truth for that quest's objective/reward/hint text. Values were identical, so no player-visible change. Behavior-preserving.</x:v>
       </x:c>
       <x:c r="AB6" t="str">
-        <x:v/>
+        <x:v>python json parse OK; validate_content passes (siege map still valid); no test references the removed config keys. Native campaign gate (siege walkthrough) confirms on CI.</x:v>
       </x:c>
       <x:c r="AC6" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>

<commit_message>
Claim s43/s44 fight-controller AI rows (level_design workbook)
- s43 EPIC_60/S02/SS04 auto-heal tempo at 75 percent HP
- s44 EPIC_60/S02/SS05 rank interactions by value not mana cost
Sequential pair (same file, both owned here). Owner controller/ctrl-vm-4039-a70f65a5.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -787,35 +787,37 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/core/CController.cpp</x:v>
       </x:c>
       <x:c r="Q9" t="str">
-        <x:v>NOT_STARTED</x:v>
+        <x:v>IN_PROGRESS</x:v>
       </x:c>
       <x:c r="R9" t="str">
-        <x:v/>
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-43</x:v>
       </x:c>
       <x:c r="S9" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="T9" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="U9"/>
-      <x:c r="V9"/>
-      <x:c r="W9"/>
+        <x:v>e7c49716-ece9-4c1b-bd7b-5228562cc07c</x:v>
+      </x:c>
+      <x:c r="U9" t="str">
+        <x:v>2026-07-03T03:57:13Z</x:v>
+      </x:c>
+      <x:c r="V9" t="str">
+        <x:v>2026-07-03T03:57:13Z</x:v>
+      </x:c>
+      <x:c r="W9" t="str">
+        <x:v>2026-07-03T07:57:13Z</x:v>
+      </x:c>
       <x:c r="X9"/>
       <x:c r="Y9" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z9" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="AA9" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="AB9" t="str">
-        <x:v/>
-      </x:c>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-43</x:v>
+      </x:c>
+      <x:c r="AA9"/>
+      <x:c r="AB9"/>
       <x:c r="AC9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -867,35 +869,37 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/core/CController.cpp</x:v>
       </x:c>
       <x:c r="Q10" t="str">
-        <x:v>NOT_STARTED</x:v>
+        <x:v>IN_PROGRESS</x:v>
       </x:c>
       <x:c r="R10" t="str">
-        <x:v/>
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-44</x:v>
       </x:c>
       <x:c r="S10" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="T10" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="U10"/>
-      <x:c r="V10"/>
-      <x:c r="W10"/>
+        <x:v>6477ddb0-6608-4317-9f5f-a250288f6658</x:v>
+      </x:c>
+      <x:c r="U10" t="str">
+        <x:v>2026-07-03T03:57:13Z</x:v>
+      </x:c>
+      <x:c r="V10" t="str">
+        <x:v>2026-07-03T03:57:13Z</x:v>
+      </x:c>
+      <x:c r="W10" t="str">
+        <x:v>2026-07-03T07:57:13Z</x:v>
+      </x:c>
       <x:c r="X10"/>
       <x:c r="Y10" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z10" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="AA10" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="AB10" t="str">
-        <x:v/>
-      </x:c>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-44</x:v>
+      </x:c>
+      <x:c r="AA10"/>
+      <x:c r="AB10"/>
       <x:c r="AC10" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Claim s43/s44 fight-controller AI rows (level_design workbook) (#1331)
- s43 EPIC_60/S02/SS04 auto-heal tempo at 75 percent HP
- s44 EPIC_60/S02/SS05 rank interactions by value not mana cost
Sequential pair (same file, both owned here). Owner controller/ctrl-vm-4039-a70f65a5.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -787,35 +787,37 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/core/CController.cpp</x:v>
       </x:c>
       <x:c r="Q9" t="str">
-        <x:v>NOT_STARTED</x:v>
+        <x:v>IN_PROGRESS</x:v>
       </x:c>
       <x:c r="R9" t="str">
-        <x:v/>
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-43</x:v>
       </x:c>
       <x:c r="S9" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="T9" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="U9"/>
-      <x:c r="V9"/>
-      <x:c r="W9"/>
+        <x:v>e7c49716-ece9-4c1b-bd7b-5228562cc07c</x:v>
+      </x:c>
+      <x:c r="U9" t="str">
+        <x:v>2026-07-03T03:57:13Z</x:v>
+      </x:c>
+      <x:c r="V9" t="str">
+        <x:v>2026-07-03T03:57:13Z</x:v>
+      </x:c>
+      <x:c r="W9" t="str">
+        <x:v>2026-07-03T07:57:13Z</x:v>
+      </x:c>
       <x:c r="X9"/>
       <x:c r="Y9" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z9" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="AA9" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="AB9" t="str">
-        <x:v/>
-      </x:c>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-43</x:v>
+      </x:c>
+      <x:c r="AA9"/>
+      <x:c r="AB9"/>
       <x:c r="AC9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -867,35 +869,37 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/core/CController.cpp</x:v>
       </x:c>
       <x:c r="Q10" t="str">
-        <x:v>NOT_STARTED</x:v>
+        <x:v>IN_PROGRESS</x:v>
       </x:c>
       <x:c r="R10" t="str">
-        <x:v/>
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-44</x:v>
       </x:c>
       <x:c r="S10" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="T10" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="U10"/>
-      <x:c r="V10"/>
-      <x:c r="W10"/>
+        <x:v>6477ddb0-6608-4317-9f5f-a250288f6658</x:v>
+      </x:c>
+      <x:c r="U10" t="str">
+        <x:v>2026-07-03T03:57:13Z</x:v>
+      </x:c>
+      <x:c r="V10" t="str">
+        <x:v>2026-07-03T03:57:13Z</x:v>
+      </x:c>
+      <x:c r="W10" t="str">
+        <x:v>2026-07-03T07:57:13Z</x:v>
+      </x:c>
       <x:c r="X10"/>
       <x:c r="Y10" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z10" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="AA10" t="str">
-        <x:v/>
-      </x:c>
-      <x:c r="AB10" t="str">
-        <x:v/>
-      </x:c>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-44</x:v>
+      </x:c>
+      <x:c r="AA10"/>
+      <x:c r="AB10"/>
       <x:c r="AC10" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Mark E60/S02/SS04 monster fight auto-heal tempo DONE (PR #1337 merged)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -787,7 +787,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/core/CController.cpp</x:v>
       </x:c>
       <x:c r="Q9" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R9" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-43</x:v>
@@ -802,20 +802,24 @@
         <x:v>2026-07-03T03:57:13Z</x:v>
       </x:c>
       <x:c r="V9" t="str">
-        <x:v>2026-07-03T03:57:13Z</x:v>
-      </x:c>
-      <x:c r="W9" t="str">
-        <x:v>2026-07-03T07:57:13Z</x:v>
-      </x:c>
-      <x:c r="X9"/>
+        <x:v>2026-07-03T04:55:20Z</x:v>
+      </x:c>
+      <x:c r="W9"/>
+      <x:c r="X9" t="str">
+        <x:v>2026-07-03T04:55:20Z</x:v>
+      </x:c>
       <x:c r="Y9" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z9" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-43</x:v>
-      </x:c>
-      <x:c r="AA9"/>
-      <x:c r="AB9"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA9" t="str">
+        <x:v>Gated CMonsterFightController auto-heal on net tempo (heal_preserves_combatant): emergency + net-gain heuristics replace the fixed 75%-HP trigger; added 3 controller unit tests. Delivered by PR #1337 (merged to main).</x:v>
+      </x:c>
+      <x:c r="AB9" t="str">
+        <x:v>PR #1337 CI green (full build + unit lanes); squash-merged to main at 6d8ee346.</x:v>
+      </x:c>
       <x:c r="AC9" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark E60/S02/SS04 monster fight auto-heal tempo DONE (PR #1337 merged) (#1345)
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -787,7 +787,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/core/CController.cpp</x:v>
       </x:c>
       <x:c r="Q9" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R9" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-43</x:v>
@@ -802,20 +802,24 @@
         <x:v>2026-07-03T03:57:13Z</x:v>
       </x:c>
       <x:c r="V9" t="str">
-        <x:v>2026-07-03T03:57:13Z</x:v>
-      </x:c>
-      <x:c r="W9" t="str">
-        <x:v>2026-07-03T07:57:13Z</x:v>
-      </x:c>
-      <x:c r="X9"/>
+        <x:v>2026-07-03T04:55:20Z</x:v>
+      </x:c>
+      <x:c r="W9"/>
+      <x:c r="X9" t="str">
+        <x:v>2026-07-03T04:55:20Z</x:v>
+      </x:c>
       <x:c r="Y9" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z9" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-43</x:v>
-      </x:c>
-      <x:c r="AA9"/>
-      <x:c r="AB9"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA9" t="str">
+        <x:v>Gated CMonsterFightController auto-heal on net tempo (heal_preserves_combatant): emergency + net-gain heuristics replace the fixed 75%-HP trigger; added 3 controller unit tests. Delivered by PR #1337 (merged to main).</x:v>
+      </x:c>
+      <x:c r="AB9" t="str">
+        <x:v>PR #1337 CI green (full build + unit lanes); squash-merged to main at 6d8ee346.</x:v>
+      </x:c>
       <x:c r="AC9" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark E60/S02/SS05 interaction ranking DONE (PR #1352 merged)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -873,7 +873,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/core/CController.cpp</x:v>
       </x:c>
       <x:c r="Q10" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R10" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-44</x:v>
@@ -888,20 +888,24 @@
         <x:v>2026-07-03T03:57:13Z</x:v>
       </x:c>
       <x:c r="V10" t="str">
-        <x:v>2026-07-03T03:57:13Z</x:v>
-      </x:c>
-      <x:c r="W10" t="str">
-        <x:v>2026-07-03T07:57:13Z</x:v>
-      </x:c>
-      <x:c r="X10"/>
+        <x:v>2026-07-03T09:06:51Z</x:v>
+      </x:c>
+      <x:c r="W10"/>
+      <x:c r="X10" t="str">
+        <x:v>2026-07-03T09:06:51Z</x:v>
+      </x:c>
       <x:c r="Y10" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z10" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-44</x:v>
-      </x:c>
-      <x:c r="AA10"/>
-      <x:c r="AB10"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA10" t="str">
+        <x:v>Replaced highest-mana interaction pick with a deterministic weakening-value ranking (expected hit + sustained opponent debuff over duration), mana affordability respected, ties toward cheaper spell. Delivered by PR #1352 (merged to main).</x:v>
+      </x:c>
+      <x:c r="AB10" t="str">
+        <x:v>PR #1352 CI green after rebase onto post-Wardens-Road main; squash-merged to main at 07:48Z.</x:v>
+      </x:c>
       <x:c r="AC10" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark E60/S02/SS05 interaction ranking DONE (PR #1352 merged) (#1359)
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_level_design_proposals.xlsx
+++ b/planning/fall_of_nouraajd_level_design_proposals.xlsx
@@ -873,7 +873,7 @@
         <x:v>https://github.com/lisu188/fall-of-nouraajd/blob/main/src/core/CController.cpp</x:v>
       </x:c>
       <x:c r="Q10" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R10" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-44</x:v>
@@ -888,20 +888,24 @@
         <x:v>2026-07-03T03:57:13Z</x:v>
       </x:c>
       <x:c r="V10" t="str">
-        <x:v>2026-07-03T03:57:13Z</x:v>
-      </x:c>
-      <x:c r="W10" t="str">
-        <x:v>2026-07-03T07:57:13Z</x:v>
-      </x:c>
-      <x:c r="X10"/>
+        <x:v>2026-07-03T09:06:51Z</x:v>
+      </x:c>
+      <x:c r="W10"/>
+      <x:c r="X10" t="str">
+        <x:v>2026-07-03T09:06:51Z</x:v>
+      </x:c>
       <x:c r="Y10" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z10" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-44</x:v>
-      </x:c>
-      <x:c r="AA10"/>
-      <x:c r="AB10"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA10" t="str">
+        <x:v>Replaced highest-mana interaction pick with a deterministic weakening-value ranking (expected hit + sustained opponent debuff over duration), mana affordability respected, ties toward cheaper spell. Delivered by PR #1352 (merged to main).</x:v>
+      </x:c>
+      <x:c r="AB10" t="str">
+        <x:v>PR #1352 CI green after rebase onto post-Wardens-Road main; squash-merged to main at 07:48Z.</x:v>
+      </x:c>
       <x:c r="AC10" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>